<commit_message>
ajout de la veille sur la rce cursor
</commit_message>
<xml_diff>
--- a/documents/Tableau-synthese-E5.xlsx
+++ b/documents/Tableau-synthese-E5.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://efrei365net-my.sharepoint.com/personal/noham_tayaa_efrei_net/Documents/BTS-SIO/Portfolio/documents/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="59" documentId="11_BDF6366FA7694CE96F0AED02F7301D2C05FF6A3B" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{13A93E94-1E29-4685-9866-7C9D6D88D905}"/>
+  <xr:revisionPtr revIDLastSave="60" documentId="11_BDF6366FA7694CE96F0AED02F7301D2C05FF6A3B" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{CCEA201B-B433-4552-9557-5DD06EFD0332}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -122,38 +122,38 @@
     <t>Mise en production de modules web en PHP MYSQL sur l'intranet</t>
   </si>
   <si>
-    <t xml:space="preserve">Recenser et identifier les ressources numérique d'un parc informatique  avec GLPI
+    <t>Déploiement d'un site web avec le service web Apache</t>
+  </si>
+  <si>
+    <t>Adresse URL du portfolio : https://n3tspy.github.io/Portfolio/</t>
+  </si>
+  <si>
+    <t>Gestion des incidents et des demandes dans GLPI</t>
+  </si>
+  <si>
+    <t>Création d'un portfolio</t>
+  </si>
+  <si>
+    <t>Mise en production de modules web sur l'intranet</t>
+  </si>
+  <si>
+    <t>Développement/amélioration de modules web PHP/MySQL sur l'intranet</t>
+  </si>
+  <si>
+    <t>Définition du cahier des charges pour le développement de modules web pour l'intranet</t>
+  </si>
+  <si>
+    <t>Traitement de tickets et demandes des collaborateurs</t>
+  </si>
+  <si>
+    <t>N° candidat : 02414309230</t>
+  </si>
+  <si>
+    <t>Période (sous la forme du 01/09/2024 au 10/05/2026)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Recensement du parc informatique avec GLPI
 </t>
-  </si>
-  <si>
-    <t>Déploiement d'un site web avec le service web Apache</t>
-  </si>
-  <si>
-    <t>Adresse URL du portfolio : https://n3tspy.github.io/Portfolio/</t>
-  </si>
-  <si>
-    <t>Gestion des incidents et des demandes dans GLPI</t>
-  </si>
-  <si>
-    <t>Création d'un portfolio</t>
-  </si>
-  <si>
-    <t>Mise en production de modules web sur l'intranet</t>
-  </si>
-  <si>
-    <t>Développement/amélioration de modules web PHP/MySQL sur l'intranet</t>
-  </si>
-  <si>
-    <t>Définition du cahier des charges pour le développement de modules web pour l'intranet</t>
-  </si>
-  <si>
-    <t>Traitement de tickets et demandes des collaborateurs</t>
-  </si>
-  <si>
-    <t>N° candidat : 02414309230</t>
-  </si>
-  <si>
-    <t>Période (sous la forme du 01/09/2024 au 10/05/2026)</t>
   </si>
 </sst>
 </file>
@@ -632,7 +632,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="164" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="47">
+  <cellXfs count="46">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
@@ -703,9 +703,48 @@
     <xf numFmtId="0" fontId="2" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -729,48 +768,6 @@
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1095,56 +1092,56 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:43" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="24" t="s">
+      <c r="A1" s="26" t="s">
         <v>7</v>
       </c>
-      <c r="B1" s="24"/>
-      <c r="C1" s="24"/>
-      <c r="D1" s="24"/>
-      <c r="E1" s="24"/>
-      <c r="F1" s="24"/>
-      <c r="G1" s="24" t="s">
+      <c r="B1" s="26"/>
+      <c r="C1" s="26"/>
+      <c r="D1" s="26"/>
+      <c r="E1" s="26"/>
+      <c r="F1" s="26"/>
+      <c r="G1" s="26" t="s">
         <v>20</v>
       </c>
-      <c r="H1" s="24"/>
+      <c r="H1" s="26"/>
     </row>
     <row r="2" spans="1:43" ht="41.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="24" t="s">
+      <c r="A2" s="26" t="s">
         <v>6</v>
       </c>
-      <c r="B2" s="24"/>
-      <c r="C2" s="24"/>
-      <c r="D2" s="24"/>
-      <c r="E2" s="24"/>
-      <c r="F2" s="24"/>
-      <c r="G2" s="24"/>
-      <c r="H2" s="24"/>
+      <c r="B2" s="26"/>
+      <c r="C2" s="26"/>
+      <c r="D2" s="26"/>
+      <c r="E2" s="26"/>
+      <c r="F2" s="26"/>
+      <c r="G2" s="26"/>
+      <c r="H2" s="26"/>
     </row>
     <row r="3" spans="1:43" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="25" t="s">
+      <c r="A3" s="38" t="s">
         <v>21</v>
       </c>
-      <c r="B3" s="26"/>
-      <c r="C3" s="26"/>
-      <c r="D3" s="26"/>
-      <c r="E3" s="27"/>
-      <c r="F3" s="31" t="s">
-        <v>35</v>
-      </c>
-      <c r="G3" s="26"/>
-      <c r="H3" s="32"/>
+      <c r="B3" s="39"/>
+      <c r="C3" s="39"/>
+      <c r="D3" s="39"/>
+      <c r="E3" s="40"/>
+      <c r="F3" s="44" t="s">
+        <v>34</v>
+      </c>
+      <c r="G3" s="39"/>
+      <c r="H3" s="45"/>
       <c r="K3" s="1"/>
       <c r="L3" s="1"/>
       <c r="M3" s="1"/>
     </row>
     <row r="4" spans="1:43" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="28" t="s">
+      <c r="A4" s="41" t="s">
         <v>22</v>
       </c>
-      <c r="B4" s="29"/>
-      <c r="C4" s="29"/>
-      <c r="D4" s="29"/>
-      <c r="E4" s="30"/>
+      <c r="B4" s="42"/>
+      <c r="C4" s="42"/>
+      <c r="D4" s="42"/>
+      <c r="E4" s="43"/>
       <c r="F4" s="14" t="s">
         <v>8</v>
       </c>
@@ -1156,23 +1153,23 @@
       </c>
     </row>
     <row r="5" spans="1:43" ht="39.9" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="43" t="s">
-        <v>28</v>
-      </c>
-      <c r="B5" s="44"/>
-      <c r="C5" s="44"/>
-      <c r="D5" s="44"/>
-      <c r="E5" s="44"/>
-      <c r="F5" s="44"/>
-      <c r="G5" s="44"/>
-      <c r="H5" s="45"/>
+      <c r="A5" s="35" t="s">
+        <v>27</v>
+      </c>
+      <c r="B5" s="36"/>
+      <c r="C5" s="36"/>
+      <c r="D5" s="36"/>
+      <c r="E5" s="36"/>
+      <c r="F5" s="36"/>
+      <c r="G5" s="36"/>
+      <c r="H5" s="37"/>
     </row>
     <row r="6" spans="1:43" ht="90" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="33" t="s">
+      <c r="A6" s="24" t="s">
         <v>17</v>
       </c>
-      <c r="B6" s="41" t="s">
-        <v>36</v>
+      <c r="B6" s="33" t="s">
+        <v>35</v>
       </c>
       <c r="C6" s="6" t="s">
         <v>0</v>
@@ -1194,8 +1191,8 @@
       </c>
     </row>
     <row r="7" spans="1:43" s="2" customFormat="1" ht="324.89999999999998" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="34"/>
-      <c r="B7" s="42"/>
+      <c r="A7" s="25"/>
+      <c r="B7" s="34"/>
       <c r="C7" s="8" t="s">
         <v>9</v>
       </c>
@@ -1251,16 +1248,16 @@
       <c r="AQ7"/>
     </row>
     <row r="8" spans="1:43" s="2" customFormat="1" ht="17.399999999999999" x14ac:dyDescent="0.25">
-      <c r="A8" s="35" t="s">
+      <c r="A8" s="27" t="s">
         <v>16</v>
       </c>
-      <c r="B8" s="36"/>
-      <c r="C8" s="36"/>
-      <c r="D8" s="36"/>
-      <c r="E8" s="36"/>
-      <c r="F8" s="36"/>
-      <c r="G8" s="36"/>
-      <c r="H8" s="37"/>
+      <c r="B8" s="28"/>
+      <c r="C8" s="28"/>
+      <c r="D8" s="28"/>
+      <c r="E8" s="28"/>
+      <c r="F8" s="28"/>
+      <c r="G8" s="28"/>
+      <c r="H8" s="29"/>
       <c r="I8"/>
       <c r="J8"/>
       <c r="K8"/>
@@ -1299,7 +1296,7 @@
     </row>
     <row r="9" spans="1:43" s="2" customFormat="1" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="11" t="s">
-        <v>26</v>
+        <v>36</v>
       </c>
       <c r="B9" s="10"/>
       <c r="C9" s="22" t="s">
@@ -1348,7 +1345,7 @@
     </row>
     <row r="10" spans="1:43" s="2" customFormat="1" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="11" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B10" s="10"/>
       <c r="C10" s="16"/>
@@ -1397,7 +1394,7 @@
     </row>
     <row r="11" spans="1:43" s="2" customFormat="1" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="11" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B11" s="10"/>
       <c r="C11" s="16"/>
@@ -1446,7 +1443,7 @@
     </row>
     <row r="12" spans="1:43" s="2" customFormat="1" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="11" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B12" s="10"/>
       <c r="C12" s="16"/>
@@ -1499,7 +1496,7 @@
       <c r="A13" s="11"/>
       <c r="B13" s="10"/>
       <c r="C13" s="16"/>
-      <c r="D13" s="46"/>
+      <c r="D13" s="16"/>
       <c r="E13" s="16"/>
       <c r="F13" s="16"/>
       <c r="G13" s="16"/>
@@ -1766,16 +1763,16 @@
       <c r="AQ18"/>
     </row>
     <row r="19" spans="1:43" s="2" customFormat="1" ht="17.399999999999999" x14ac:dyDescent="0.25">
-      <c r="A19" s="38" t="s">
+      <c r="A19" s="30" t="s">
         <v>18</v>
       </c>
-      <c r="B19" s="39"/>
-      <c r="C19" s="39"/>
-      <c r="D19" s="39"/>
-      <c r="E19" s="39"/>
-      <c r="F19" s="39"/>
-      <c r="G19" s="39"/>
-      <c r="H19" s="40"/>
+      <c r="B19" s="31"/>
+      <c r="C19" s="31"/>
+      <c r="D19" s="31"/>
+      <c r="E19" s="31"/>
+      <c r="F19" s="31"/>
+      <c r="G19" s="31"/>
+      <c r="H19" s="32"/>
       <c r="I19"/>
       <c r="J19"/>
       <c r="K19"/>
@@ -1814,7 +1811,7 @@
     </row>
     <row r="20" spans="1:43" s="2" customFormat="1" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="11" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B20" s="10"/>
       <c r="C20" s="16"/>
@@ -1863,7 +1860,7 @@
     </row>
     <row r="21" spans="1:43" s="2" customFormat="1" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="21" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B21" s="10"/>
       <c r="C21" s="22" t="s">
@@ -1914,7 +1911,7 @@
     </row>
     <row r="22" spans="1:43" s="2" customFormat="1" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="11" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B22" s="10"/>
       <c r="C22" s="16"/>
@@ -2142,16 +2139,16 @@
       <c r="AQ26"/>
     </row>
     <row r="27" spans="1:43" s="2" customFormat="1" ht="17.399999999999999" x14ac:dyDescent="0.25">
-      <c r="A27" s="38" t="s">
+      <c r="A27" s="30" t="s">
         <v>19</v>
       </c>
-      <c r="B27" s="39"/>
-      <c r="C27" s="39"/>
-      <c r="D27" s="39"/>
-      <c r="E27" s="39"/>
-      <c r="F27" s="39"/>
-      <c r="G27" s="39"/>
-      <c r="H27" s="40"/>
+      <c r="B27" s="31"/>
+      <c r="C27" s="31"/>
+      <c r="D27" s="31"/>
+      <c r="E27" s="31"/>
+      <c r="F27" s="31"/>
+      <c r="G27" s="31"/>
+      <c r="H27" s="32"/>
       <c r="I27"/>
       <c r="J27"/>
       <c r="K27"/>
@@ -2239,7 +2236,7 @@
     </row>
     <row r="29" spans="1:43" s="2" customFormat="1" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" s="11" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B29" s="10"/>
       <c r="C29" s="16"/>
@@ -2288,7 +2285,7 @@
     </row>
     <row r="30" spans="1:43" s="2" customFormat="1" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A30" s="11" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B30" s="10"/>
       <c r="C30" s="22" t="s">
@@ -2610,6 +2607,11 @@
     <row r="81" customFormat="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <mergeCells count="12">
+    <mergeCell ref="G1:H1"/>
+    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A3:E3"/>
+    <mergeCell ref="A4:E4"/>
+    <mergeCell ref="F3:H3"/>
     <mergeCell ref="A6:A7"/>
     <mergeCell ref="A2:H2"/>
     <mergeCell ref="A8:H8"/>
@@ -2617,11 +2619,6 @@
     <mergeCell ref="A27:H27"/>
     <mergeCell ref="B6:B7"/>
     <mergeCell ref="A5:H5"/>
-    <mergeCell ref="G1:H1"/>
-    <mergeCell ref="A1:F1"/>
-    <mergeCell ref="A3:E3"/>
-    <mergeCell ref="A4:E4"/>
-    <mergeCell ref="F3:H3"/>
   </mergeCells>
   <phoneticPr fontId="2" type="noConversion"/>
   <printOptions horizontalCentered="1" verticalCentered="1"/>

</xml_diff>